<commit_message>
Update fixture xlsx templates: rename 수준 header to 부문
Keeps templates in sync with the app's required roster column name.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/대진표_예시.xlsx
+++ b/fixtures/대진표_예시.xlsx
@@ -399,17 +399,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E13"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>수준</v>
+        <v>부문</v>
       </c>
       <c r="B1" t="str">
         <v>조</v>
@@ -638,11 +631,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C14"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="80.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>